<commit_message>
Auto sync live sales control data with HKT timezone fix and reverse sold auto-correction: 2026-08-01 11:37:04
</commit_message>
<xml_diff>
--- a/files/九龙-九龙塘-Park College.xlsx
+++ b/files/九龙-九龙塘-Park College.xlsx
@@ -764,7 +764,7 @@
       </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
-          <t>2026-01-20</t>
+          <t>2026-01-21</t>
         </is>
       </c>
       <c r="H3" s="5" t="n">
@@ -830,7 +830,7 @@
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>2026-04-20</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="H4" s="5" t="n">
@@ -896,7 +896,7 @@
       </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="H5" s="5" t="n">
@@ -962,7 +962,7 @@
       </c>
       <c r="G6" s="3" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-28</t>
         </is>
       </c>
       <c r="H6" s="5" t="n">
@@ -1028,7 +1028,7 @@
       </c>
       <c r="G7" s="3" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="H7" s="5" t="n">
@@ -1094,7 +1094,7 @@
       </c>
       <c r="G8" s="3" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="H8" s="5" t="n">
@@ -1230,7 +1230,7 @@
       </c>
       <c r="G10" s="3" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="H10" s="5" t="n">
@@ -1296,7 +1296,7 @@
       </c>
       <c r="G11" s="3" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="H11" s="5" t="n">
@@ -1362,7 +1362,7 @@
       </c>
       <c r="G12" s="3" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="H12" s="5" t="n">
@@ -1595,7 +1595,7 @@
           <t>A | 3040呎 (4+房)
 $12800万
 $42,105/呎
-(26年-04月-20日)</t>
+(26年-04月-21日)</t>
         </is>
       </c>
       <c r="C5" s="20" t="inlineStr">
@@ -1603,7 +1603,7 @@
           <t>B | 3022呎 (4+房)
 $15000万
 $49,636/呎
-(26年-01月-20日)</t>
+(26年-01月-21日)</t>
         </is>
       </c>
       <c r="D5" s="21" t="inlineStr"/>
@@ -1619,7 +1619,7 @@
           <t>A | 1478呎 (3房)
 $6000万
 $40,595/呎
-(26年-05月-27日)</t>
+(26年-05月-28日)</t>
         </is>
       </c>
       <c r="C6" s="20" t="inlineStr">
@@ -1627,7 +1627,7 @@
           <t>B | 1463呎 (3房)
 $6000万
 $41,012/呎
-(26年-05月-27日)</t>
+(26年-05月-28日)</t>
         </is>
       </c>
       <c r="D6" s="21" t="inlineStr"/>
@@ -1643,7 +1643,7 @@
           <t>A | 1478呎 (3房)
 $5900万
 $39,919/呎
-(26年-06月-22日)</t>
+(26年-06月-23日)</t>
         </is>
       </c>
       <c r="C7" s="20" t="inlineStr">
@@ -1651,7 +1651,7 @@
           <t>B | 1463呎 (3房)
 $5900万
 $40,328/呎
-(26年-06月-22日)</t>
+(26年-06月-23日)</t>
         </is>
       </c>
       <c r="D7" s="21" t="inlineStr"/>
@@ -1667,7 +1667,7 @@
           <t>A | 1478呎 (3房)
 $6000万
 $40,595/呎
-(26年-06月-28日)</t>
+(26年-06月-29日)</t>
         </is>
       </c>
       <c r="C8" s="22" t="inlineStr">
@@ -1691,7 +1691,7 @@
           <t>A | 1405呎 (3房)
 $6300万
 $44,840/呎
-(26年-06月-22日)</t>
+(26年-06月-23日)</t>
         </is>
       </c>
       <c r="C9" s="20" t="inlineStr">
@@ -1699,7 +1699,7 @@
           <t>B | 1390呎 (3房)
 $6000万
 $43,165/呎
-(26年-06月-22日)</t>
+(26年-06月-23日)</t>
         </is>
       </c>
       <c r="D9" s="21" t="inlineStr"/>

</xml_diff>